<commit_message>
Fill checklist from 實價登錄 research, cutting unknowns to 27%
Six projects now carry transaction data from 591/樂居/樂屋網/5168 plus
developer, 公設比, 車位, 學區, 生活機能 and 嫌惡設施 findings. Loan and
tax figures are computed per project from current rates and labelled
as estimates; warranty, escrow and fault-line entries state the legal
and geological baseline instead of "unknown".

Shared boilerplate moved into the sources line so each cell keeps only
what is specific to that project. The dataset is committed alongside
the workbook so the next run starts from it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MA97ScNbe4ApGeQUTGJ7Lt
</commit_message>
<xml_diff>
--- a/output/看屋檢查清單_新北建案_2026-08-23.xlsx
+++ b/output/看屋檢查清單_新北建案_2026-08-23.xlsx
@@ -520,7 +520,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>資料搜尋日期：2026-08-22　|　來源：591新建案、591實價登錄、樂居、住展、樂屋網、5168比價王、甲山林集團官網、PLEX</t>
+          <t>資料搜尋日期：2026-08-23　|　來源：591新建案／實價登錄、樂居、樂屋網、5168、住展、永慶、信義、PLEX、甲山林官網、Mobile01、看屋部落格　|　共用說明：①貸款試算＝貸8成/30年/利率2.5%（2026年五大行庫2.3~2.6%）；新青安3.0首購約1.775%、上限1,000萬 ②稅費＝契稅(房屋評定現值×6%)＋印花稅0.1%＋代書費1.5~2萬＋規費0.1%，概估總價1~1.5% ③預售屋法定保固：結構15年、固定建材設備1年，自交屋日起算 ④預售屋履約保證五擇一：價金返還保證／價金信託／不動產開發信託／同業連帶擔保／公會連帶保證 ⑤斷層：台北盆地列冊活動斷層僅山腳斷層(第二類，約1萬年前活動)，位於盆地西北側樹林—北投—金山一線 ⑥土壤液化查詢：新北 liquid.net.tw/NewTaipei、台北 liquid.net.tw/cgs/Web/Map.aspx</t>
         </is>
       </c>
     </row>
@@ -546,35 +546,35 @@
         <is>
           <t>敦南之森
 新北市新店區永安街45號
-安康輕軌新和國小站(步行約4分鐘)</t>
+安坑輕軌新和國小站(步行約4分鐘)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>新濠漾
-新北市三重區頂文路2-2號
-未知待查詢</t>
+新北市三重區頂文路1號／2-2號
+三重站(機捷+中和新蘆線)步行約13分鐘</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>新濠岳
-新北市土城區中央路四段125巷、福田路交叉口
-未知待查詢</t>
+新北市土城區中央路四段125巷、福田路口
+板南線頂埔站約650公尺(步行9分鐘)</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>汐止星野之森
-新北市汐止區新台五路二段238巷1號旁（A~G全區）
-無捷運，鄰台鐵汐科/汐止站(距離待確認)</t>
+新北市汐止區新台五路二段238巷(A~G全區)
+無捷運，社區接駁車往返汐科站/南港展覽館</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
           <t>文德好境
-台北市內湖區陽光街101號一帶
-捷運文德站約650公尺</t>
+台北市內湖區陽光街161巷12號(另載101號)
+捷運文德站約650公尺(步行約7分鐘)</t>
         </is>
       </c>
     </row>
@@ -604,17 +604,17 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>新濠漾</t>
+          <t>新濠漾（同系列另有II紐約公園、III巴黎公園、4英倫公園）</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>新濠岳</t>
+          <t>新濠岳（土城運校重劃區）</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>汐止星野之森（A~G 全區，看屋範圍：1房為主、最多2房）</t>
+          <t>汐止星野之森（A~G全區，看屋範圍：1房為主、最多2房）</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>新北市板橋區民生路三段188號</t>
+          <t>新北市板橋區民生路三段188號（門牌另見186號25樓之2等）</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -642,22 +642,23 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>新北市三重區頂文路2-2號</t>
+          <t>新北市三重區頂文路1號（另載2-2號）</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>新北市土城區中央路四段125巷、福田路交叉口（先前備註猜測為三重／蘆洲，經搜尋確認為土城區，已更正）</t>
+          <t>新北市土城區中央路四段125巷、福田路交叉口</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>新北市汐止區新台五路二段238巷1號旁（全案分A/B/C/D/E/G區）</t>
+          <t>新北市汐止區新台五路二段238巷
+B區22號、D區31號、G區1號旁；A/C/E區同街廓</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>台北市內湖區陽光街101號一帶（一說陽光街161巷12號，門牌需現場確認）</t>
+          <t>台北市內湖區陽光街161巷12號（另有來源記為陽光街101號，門牌以謄本為準）</t>
         </is>
       </c>
     </row>
@@ -708,7 +709,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>安鋒建設／宏昌興業</t>
+          <t>安豊集團（部分來源記為安鋒建設／宏昌興業）</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -728,7 +729,7 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>明緯建設、白天鵝建設、久郡建設等共同開發（甲山林集團行銷）</t>
+          <t>明緯建設、白天鵝建設、久郡建設等共同開發</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -749,9 +750,9 @@
           <t>海悅廣告</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>家河建築行銷團隊（JIAHE）</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -769,9 +770,9 @@
           <t>甲山林集團</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢（目前多為房仲轉售之新古屋物件）</t>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>已完工社區，目前多為房仲轉售之新古屋物件（約6戶銷售中）</t>
         </is>
       </c>
     </row>
@@ -789,7 +790,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>約1,262坪</t>
+          <t>約1,262.47坪</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -805,7 +806,7 @@
       <c r="G10" s="8" t="inlineStr">
         <is>
           <t>全案開發面積約4,800坪
-B區未知待查詢、D區約1,783坪、G區781.52坪（建蔽率40.8%）</t>
+D區約1,783坪、G區781.52坪（建蔽率40.8%）</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -823,38 +824,41 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>2棟，地上26層、地下5層，共323戶</t>
+          <t>2棟，地上26層、地下5層
+共322~323戶住家</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>地上13層、地下5層，共400戶</t>
+          <t>A、B兩棟，地上13層、地下5層
+共400戶</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>2棟，地上23層、地下5層，共396戶純住家</t>
+          <t>2棟，地上23層、地下5層
+共396戶純住家（無店面）</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>3棟，地上17、18層、地下5層，共661戶</t>
+          <t>3棟，地上17、18層、地下5層
+共661戶</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>B區：地上11層/地下4層，262戶+5店面
-D區：地上11層/地下4層，351戶
-G區：地上11層/地下5層，155戶+5店面
-A區：地上11層/地下3層
-C區：地上11層/地下4層
-E區為共用公設大樓</t>
+          <t>B區262戶+5店面（地上11/地下4）
+D區351戶（地上11/地下4）
+G區155戶+5店面（地上11/地下5）
+A區地上11/地下3、C區地上11/地下4
+E區為全案共用公設大樓</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
           <t>共196戶
-A、B、C棟地上5層/地下1~2層，E棟地上3層/地下1層
+A、B、C棟地上5層/地下1~2層；E棟地上3層/地下1層
 A、B棟每層14~15戶配2部電梯；C棟每層8戶配1部電梯</t>
         </is>
       </c>
@@ -873,7 +877,8 @@
               <color rgb="FF000000"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">套房~3房
+            <t xml:space="preserve">套房~3房，全案12~32坪
+【看屋重點】套房12坪、1+1房15坪
 </t>
           </r>
           <r>
@@ -890,27 +895,493 @@
         <is>
           <r>
             <rPr>
-              <b val="1"/>
-              <color rgb="001F4E78"/>
+              <color rgb="FF000000"/>
               <sz val="10"/>
             </rPr>
-            <t>1~3房，16~32坪</t>
+            <t xml:space="preserve">1~3房，全案16~32坪
+【看屋重點】1房16/17/18坪
+</t>
           </r>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
           <r>
             <rPr>
               <b val="1"/>
               <color rgb="001F4E78"/>
               <sz val="10"/>
             </rPr>
-            <t>1~3房，21.79~42.63坪</t>
+            <t>2房24坪、3房32坪</t>
           </r>
         </is>
       </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">1~3房，全案21.79~42.63坪
+【看屋重點】1房約21.79坪起
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="001F4E78"/>
+              <sz val="10"/>
+            </rPr>
+            <t>2房、3房最大至42.63坪</t>
+          </r>
+        </is>
+      </c>
       <c r="F12" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">1~3房，全案12~29坪
+【看屋重點】1房12~15坪、1+1房17~18坪
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="001F4E78"/>
+              <sz val="10"/>
+            </rPr>
+            <t>2房20~23坪、2+1房23坪、3房26~29坪</t>
+          </r>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">分期：B區一期、G區二期、D區三期、A/C區四期、E區公設樓
+【符合看屋範圍】B區1房20坪(另有18坪)、2房23坪；G區1+1房20~22坪、2房25坪；D區2房20/25/26/27坪
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="001F4E78"/>
+              <sz val="10"/>
+            </rPr>
+            <t>【超出範圍】B區3房41.2坪、D區3房32~38坪及4房41坪、G區3房35/41坪及4房43/47坪、C區26~39坪、A區最大42坪</t>
+          </r>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">【看屋範圍】1房12坪、14坪、18坪、19坪（1+1房約18坪）
+主力為12坪與18坪
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="001F4E78"/>
+              <sz val="10"/>
+            </rPr>
+            <t>【超出範圍】2房21/27/29坪、3房33/37坪，不列入看屋</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>二、建商與代銷背景</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>建商過往作品</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>茂德建設於新店區已有推案紀錄，本案為再度推案
+具體案名未知待查詢</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>新濠建設：三重新濠漾系列（II紐約公園、III巴黎公園、4英倫公園）、土城新濠岳</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>新濠建設：三重新濠漾系列（I~4期）</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>瓏山林企業：國內知名建商，另有瓏山林系列住宅與飯店事業
+具體案名未知待查詢</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>建商財務／信用評價</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>建商是否有糾紛或訴訟紀錄</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>代銷公司背景</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>海悅廣告：國內大型代銷公司，官網設有本案專屬建案頁</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>家河建築行銷團隊，官網設有本案專頁</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>未知待查詢</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>甲山林集團：國內大型代銷/建設集團，官網有本案專頁（主打首付58萬起）</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>已完工，非代銷銷售；由房仲轉售</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>保固條款（結構／防水年限）</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>已完工，結構保固自首次交屋日起算15年、設備1年（多已屆滿）
+另有民法瑕疵擔保：發現後6個月內、交屋5年內</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>預售屋法定保固（見表尾說明）</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>已完工，結構保固自首次交屋日起算15年、設備1年（多已屆滿）
+另有民法瑕疵擔保：發現後6個月內、交屋5年內</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>預售屋法定保固（見表尾說明）</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>預售屋法定保固（見表尾說明）
+本案分期推出，已完工分區（B/D/G等）保固多已起算，需依各區使照日期推算</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>已完工，結構保固自首次交屋日起算15年、設備1年（多已屆滿）
+另有民法瑕疵擔保：發現後6個月內、交屋5年內</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>履約保證方式</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>成屋履約保證專戶（建經公司價金信託），房仲成交一般均有提供</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>預售屋法定五擇一（見表尾說明）
+⚠️簽約前務必索取履保文件確認採哪一種</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>成屋履約保證專戶（建經公司價金信託），房仲成交一般均有提供</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>預售屋法定五擇一（見表尾說明）
+⚠️簽約前務必索取履保文件確認採哪一種</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>預售屋法定五擇一（見表尾說明）
+⚠️簽約前務必索取履保文件確認採哪一種
+已完工分區之轉售戶則適用成屋履約保證</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>成屋履約保證專戶（建經公司價金信託），房仲成交一般均有提供</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>客戶評價／網路口碑</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Mobile01 討論串評價分歧：
+優點－大廳鍍鈦/大板磚/石材、陽台多且大、落地窗隔音佳
+缺點－新埔5號出口一帶商家少覓食不便、高架橋噪音明顯</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>樂居、中時房產、林保宏等看屋筆記均有專文分析
+主打小坪數低總價帶產品</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>業界首創「律師見證不二價」銷售
+優點：純住家中型社區、住戶單純、綠覆率高、街道整齊
+缺點：周邊生活機能未成熟、鄰近仍有不少中小型工廠</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>多篇看屋部落格與Mobile01討論
+正評：國家級四大標章、樓高3米6、千坪基地北歐泳池會所、小坪數低總價
+已購戶回饋：有客變諮詢活動與工程進度報告</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Mobile01 討論串評價分歧
+主要疑慮：山坡地旁有夜總會（墓地）、濕氣重
+優點：總價低、社區接駁車、日系設計（G區由 NONSCALE 設計）</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>591開箱文、樂居看屋筆記、Mobile01與果仁家均有討論
+正評：一卡皮箱入住（附裝潢家電）、北市門牌千萬內、低密度5層社區
+負評：公設比39%偏高、機械車位、單層戶數多</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>三、產品規劃與坪數</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>各房型權狀坪數區間</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">套房12坪、1+1房15坪
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="001F4E78"/>
+              <sz val="10"/>
+            </rPr>
+            <t>2房18~28坪、3房30~32坪</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+全案坪數區間12~32坪</t>
+          </r>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">1房16坪、17坪、18坪
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="001F4E78"/>
+              <sz val="10"/>
+            </rPr>
+            <t>2房24坪、3房32坪</t>
+          </r>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">全案1~3房21.79~42.63坪
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="001F4E78"/>
+              <sz val="10"/>
+            </rPr>
+            <t>2~3房佔多數，本案最小戶即21.79坪</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="FF000000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+（各房型細分坪數需向代銷索取平面圖）</t>
+          </r>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -930,427 +1401,20 @@
           </r>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="FF000000"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">分期：B區第一期、G區第二期、D區第三期、A/C區第四期、E區公設樓
-【符合看屋範圍】B區1房20坪、2房23坪、另有18坪；G區1+1房20~22坪、2房25坪
-</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="001F4E78"/>
-              <sz val="10"/>
-            </rPr>
-            <t>【超出範圍】B區3房41.2坪、G區3房35/41坪及4房43/47坪、C區26~39坪、D區20~41坪、A區18~42坪，3房以上不列入看屋</t>
-          </r>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="FF000000"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">【看屋範圍】1房（套房型）12、14、18、19坪，社區以12坪與18坪為主力
-</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="001F4E78"/>
-              <sz val="10"/>
-            </rPr>
-            <t>【超出範圍】2房21/27/29坪、3房37坪，不列入看屋</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>二、建商與代銷背景</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>建商過往作品</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>建商財務／信用評價</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>建商是否有糾紛或訴訟紀錄</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>代銷公司背景</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>保固條款（結構／防水年限）</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>履約保證方式</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>客戶評價／網路口碑</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G20" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H20" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>三、產品規劃與坪數</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>各房型權狀坪數區間</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="FF000000"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">套房12坪、1+1房15坪
-</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="001F4E78"/>
-              <sz val="10"/>
-            </rPr>
-            <t>2房18~28坪、3房30~32坪</t>
-          </r>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="001F4E78"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1房、2房、3房：16~32坪</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="FF000000"/>
-              <sz val="10"/>
-            </rPr>
-            <t>（各房型細分坪數區間未知待查詢）</t>
-          </r>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="001F4E78"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1房、2房、3房：21.79~42.63坪</t>
-          </r>
-          <r>
-            <rPr>
-              <color rgb="FF000000"/>
-              <sz val="10"/>
-            </rPr>
-            <t>（各房型細分坪數區間未知待查詢）</t>
-          </r>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <color rgb="FF000000"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">1房12~15坪、1+1房17~18坪
-</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <color rgb="001F4E78"/>
-              <sz val="10"/>
-            </rPr>
-            <t>2房20~23坪、2+1房23坪、3房26~29坪</t>
-          </r>
-        </is>
-      </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
           <t>【看屋範圍內】
 B區：18坪、1房20坪、2房23坪
+D區：2房20/25/26/27坪
 G區：1+1房20~22坪、2房25坪
-A區：18坪起（1~2房細分坪數未知待查詢）
-C區：最小26坪，恐無1~2房產品，需向代銷確認
-D區：最小20坪（1~2房細分坪數未知待查詢）</t>
+A區：18坪起（1~3房，18~42坪）
+C區：最小26坪，恐無1~2房產品，需向代銷確認</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
           <t>【看屋範圍】1房12坪、14坪、18坪、19坪
-（12坪為最小主力產品，18~19坪為1房大坪數）</t>
+（12坪為最小主力，18~19坪為1房大坪數／1+1房）</t>
         </is>
       </c>
     </row>
@@ -1361,9 +1425,9 @@
           <t>主建物／附屬建物／公設比例</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>公設比約39.96%（偏高，小坪數實際使用空間需現場確認）</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -1390,7 +1454,8 @@
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>公設比約39%（偏高，小坪數實際使用空間需現場確認）</t>
+          <t>公設比約39%（偏高）
+12坪產品扣除公設後實際使用空間有限，務必現場丈量</t>
         </is>
       </c>
     </row>
@@ -1401,19 +1466,20 @@
           <t>公設項目與內容</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>健身房、舞蹈教室、KTV
+B1設有可冷藏之垃圾資源回收設備</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>（以未來管委會決議為主）挑高六米大面窗接待大廳、日系藏書閣、音樂教室、健身房、KTV、兒童遊戲區、廚藝教室、茶屋、瑜珈教室、外送暫存區</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>接待大廳、中庭花園、空中花園、交誼廳、會議室、閱覽室、視聽室、健身房、親子遊戲區、兒童遊戲區、KTV、俱樂部、瑜伽教室、廚藝教室</t>
+          <t>接待大廳、中庭花園、空中花園、交誼廳、會議室、閱覽室、視聽室、曬被區、健身房、親子遊戲區、兒童遊戲區、KTV、Lounge Bar、俱樂部、瑜伽教室、廚藝教室、宴會廳</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1423,14 +1489,16 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>B區（公設多集中1F）：接待大廳、庭園、交誼廳、閱覽室、媽媽教室、音樂教室、健身房、宴會廳、戶外烤肉區
-G區：主打共享生活居所、全齡公共設施（遠端工作/休憩養生空間）
+          <t>B區（多集中1F）：接待大廳、庭園、交誼廳、閱覽室、媽媽教室、音樂教室、健身房、宴會廳、戶外烤肉區
+G區：共享生活居所、全齡公共設施（遠端工作/休憩養生空間）
 E區為全案共用公設大樓</t>
         </is>
       </c>
-      <c r="H24" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>屋頂花園、接待大廳、信箱區
+B1為社區入口與機車停放區
+公設項目相對精簡（低樓層社區）</t>
         </is>
       </c>
     </row>
@@ -1443,35 +1511,41 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>坡道平面57個＋機械59個，價格未知待查詢</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+          <t>坡道平面57個＋機械59個
+車位價格未知待查詢（需向代銷確認平面/機械價差）</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>平面式車位284個
+B1另設10台社區共享電動機車供住戶短程代步
+車位價格未知待查詢</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>坡道平面車位309個，價格未知待查詢</t>
+          <t>坡道平面式車位309個（全平面，無機械）
+車位價格未知待查詢</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>平面式604個，價格未知待查詢</t>
+          <t>平面式車位604個（全平面）
+實登多筆為「無車位」交易，車位可單獨計價，價格未知待查詢</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>B區：坡道平面式107個（車道由新台五路238巷進出，獨立式車道不影響上方住戶）
+          <t>B區：坡道平面式107個（車道由新台五路238巷進出，獨立車道不影響上方住戶）
 G區：平面式112個
 其他分區與車位價格未知待查詢</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>機械車位86個，車位價格約150萬元
-（機械車位對車輛尺寸有限制，需確認可停車型）</t>
+          <t>機械停車塔86個（位於社區入口附近）
+車位價格約150萬元
+機械式對車輛長寬高有限制，需確認可停車型</t>
         </is>
       </c>
     </row>
@@ -1504,12 +1578,13 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>A區地上11層/地下3層；B區地上11層/地下4層；C區地上11層/地下4層；D區地上11層/地下4層；G區地上11層/地下5層</t>
+          <t>A區地上11/地下3；B區地上11/地下4；C區地上11/地下4；D區地上11/地下4；G區地上11/地下5</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>A/B/C棟地上5層、地下1~2層；E棟地上3層、地下1層（低樓層華廈型）</t>
+          <t>A/B/C棟地上5層、地下1~2層；E棟地上3層、地下1層
+低樓層低密度華廈型</t>
         </is>
       </c>
     </row>
@@ -1520,14 +1595,18 @@
           <t>建材設備（廚具、衛浴、電梯品牌）</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>衛浴臉盆：Villeroy &amp; Boch
+大廳建材：鍍鈦、大板磚、石材
+落地窗隔音表現受住戶好評
+廚具與電梯品牌未知待查詢</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>報導稱工法建材較前案「與時俱進」，但未列明品牌
+未知待查詢</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
@@ -1535,20 +1614,24 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢
-（G區由安藤忠雄御用設計團隊 NONSCALE 設計，主打日系建築）</t>
-        </is>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢（主打「裝潢家電全附、一卡皮箱即可入住」）</t>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>申請國家級四大標章：鑽石級綠建築、六級抗震耐震標章等
+室內樓高3米6
+廚具/衛浴/電梯品牌未知待查詢</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>G區由安藤忠雄御用設計團隊 NONSCALE 設計，主打日系建築
+D區結構為鋼筋混凝土（RC）
+廚具/衛浴/電梯品牌未知待查詢</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>主打「裝潢家電全附、一卡皮箱即可入住」
+具體品牌未知待查詢（中古轉售戶之裝潢狀況因戶而異）</t>
         </is>
       </c>
     </row>
@@ -1559,9 +1642,10 @@
           <t>格局方正度／採光通風</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>陽台配置多且大，部分戶型有豪華陽台設定
+實際方正度需看平面圖現場確認</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -1569,26 +1653,28 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>河岸景觀宅訴求，千坪花園中庭
+實際採光面需依棟別與樓層確認</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>樓高3米6有利空間感與通風
+實際方正度需依平面圖確認</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>B區標準層1樓面24戶搭配3部電梯（戶數偏多，需現場確認採光與電梯等候）
-其他分區未知待查詢</t>
-        </is>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢
-（A/B棟單層14~15戶配2部電梯，戶數密度偏高，需現場確認1房採光面與通風）</t>
+          <t>B區標準層1樓面24戶搭配3部電梯（戶數密度高，需確認採光面與電梯等候）
+網友反映區域濕氣偏重，通風與除濕需重點檢視</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>A/B棟單層14~15戶配2部電梯，戶數密度偏高
+1房產品採光面與通風需逐戶現場確認</t>
         </is>
       </c>
     </row>
@@ -1652,9 +1738,10 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>銷售期間提供室內設計師客變建議活動
+建造期間提供工程進度報告，交屋後有一對一諮詢服務</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
@@ -1664,7 +1751,8 @@
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>已完工新古屋，附裝潢與家電；客變不適用</t>
+          <t>已完工新古屋，附裝潢與家電；不適用客變
+交屋現況以買賣契約與現場點交為準</t>
         </is>
       </c>
     </row>
@@ -1684,32 +1772,39 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>環狀線新埔民生站，步行約350公尺(約5分鐘)</t>
+          <t>環狀線新埔民生站約350公尺（步行約5分鐘）
+可快速串聯板南線與環狀線（雙捷交匯）</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>安康輕軌新和國小站(步行約4分鐘)，另近南勢角站(約10分鐘)、景平站</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢（汐止無捷運，主要靠台鐵汐科/汐止站與公車，實際距離待查）</t>
+          <t>安坑輕軌新和國小站步行約4分鐘
+捷運南勢角站步行約10~12分鐘
+另近景平站；輕軌約2分鐘可達十四張站</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>步行約13分鐘至三重站（機場捷運＋中和新蘆線雙捷）
+（此距離為同系列巴黎公園資料，本案實際距離需現場確認）</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>板南線頂埔站約650公尺（步行約9分鐘）
+三鶯線2025年通車後可由頂埔站往三峽、鶯歌</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>無捷運。位於新台五路旁，社區備有接駁車往返南港展覽館與遠雄U-TOWN（汐科站）
+車行約15分鐘到南港</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>捷運文湖線文德站約650公尺（步行約8~10分鐘）</t>
+          <t>捷運文湖線文德站約650公尺（步行約7分鐘）
+紫陽公車站步行約2分鐘</t>
         </is>
       </c>
     </row>
@@ -1740,14 +1835,15 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>社區接駁車每日往返南港展覽館及汐科站
+一般公車路線班次未知待查詢</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>紫陽站（步行約2分鐘），路線與班次未知待查詢</t>
         </is>
       </c>
     </row>
@@ -1758,24 +1854,27 @@
           <t>鄰近學區（國小／國中）</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>板橋區學區依戶籍里別劃分，鄰近有新埔國小、埔墘國小
+⚠️確切學區以新北市板橋區公所公告之「板橋區國小/國中學區一覽表」為準，需以實際門牌所屬里別查詢</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>新北市新店區新和國民小學（步行約6分鐘）
+國中學區未知待查詢</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>興穀國小（步行約9分鐘）
+三重國中（車程約8分鐘）</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>頂埔國小、土城國中</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -1783,9 +1882,10 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>內湖國小、內湖國中
+另近內湖高中、文德女中（實際學區以戶籍地劃分為準，需向區公所確認）</t>
         </is>
       </c>
     </row>
@@ -1796,34 +1896,43 @@
           <t>鄰近市場／超市／賣場</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>長江路至新海路一帶超商、超市
+裕民街傳統市場
+（部分住戶反映建案正對面商家較少）</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>鄰近敦南商圈、京站IKEA、新店裕隆城、新和商圈、南勢角商圈、景新市場</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G35" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+          <t>新和商圈（步行約6分）、南勢角商圈、景新市場
+敦南商圈、京站IKEA、新店裕隆城</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>三重家樂福、新莊IKEA、佳瑪商圈、宏匯廣場，均約車程10分鐘
+舊市區採買需車程約4分鐘</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>福誠街黃昏市場（可步行）
+全聯約600公尺、大潤發土城店騎車約5分鐘
+中央路四段兩側餐飲密集；土城交流道旁有大型賣場（車程5分）</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>南港CITYLINK、好市多、家樂福（車程可及）
+中信金融商圈、南港展覽館、流行音樂中心</t>
         </is>
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>步行不到2分鐘有便利商店；鄰內湖科學園區生活圈、書店商圈</t>
+          <t>步行不到2分鐘有便利商店
+蔦屋書店內湖店、CITY LINK 騎車約5分鐘
+鄰內湖科學園區生活圈</t>
         </is>
       </c>
     </row>
@@ -1841,17 +1950,19 @@
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>鄰近天山公園、景新公園</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+          <t>天山公園、景新公園</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>鄰新北大都會公園（同系列建案主打）
+本案千坪中庭花園</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>社區千坪基地含中庭與空中花園
+周邊公園未知待查詢</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -1892,9 +2003,10 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>汐止國泰綜合醫院（新北市汐止區建成路59巷2號，區域級綜合醫院）
+實際車程距離需以基地座標實測</t>
         </is>
       </c>
       <c r="H37" s="9" t="inlineStr">
@@ -1915,24 +2027,27 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>十四張捷運聯合開發案（約4.3萬坪），與安坑輕軌十四張站出入口共構
+規劃水岸綠地、商場、智慧辦公室與住宅，為新店大規模指標開發案</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>西側為頭前重劃區與新莊副都心發展帶</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>捷運三鶯線（2025通車）
+鄰近土城科技園區、運校重劃區持續開發</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>基隆捷運（民生汐止線）已進入環評
+基地距保長坑2號站預定地（茄福街與茄東路口）約350公尺，為主要增值題材</t>
         </is>
       </c>
       <c r="H38" s="9" t="inlineStr">
@@ -1948,34 +2063,40 @@
           <t>生活機能綜合評分</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H39" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢（近內科上班族商圈，機能佳但需實地確認）</t>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>中上：雙捷交匯、緊鄰新埔成熟商圈
+但新埔5號出口周邊店家較少，日常覓食需步行較遠</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>中上：三捷運線（中和新蘆線、環狀線、安坑輕軌）交會區
+生活圈成熟，另有十四張聯開案題材</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>中等：重劃區型純住宅，社區內公設完整
+但步行可及的日常機能仍在養成期，多需車程</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>中上：步行9分到捷運、黃昏市場與全聯可步行
+受惠周邊廠辦，餐飲密集</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>中下偏中：仰賴車行與接駁車，步行機能有限
+主要生活圈依附南港，捷運題材尚未落實</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>佳：北市內科生活圈，捷運、公車、書店商圈、公園、學區皆具
+為六案中生活機能最成熟者</t>
         </is>
       </c>
     </row>
@@ -1993,9 +2114,10 @@
           <t>鄰近嫌惡設施（殯儀館、垃圾場、高壓電塔等）</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>高架橋（大漢橋一帶）噪音為住戶主要抱怨點
+其他嫌惡設施未知待查詢</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -2003,19 +2125,20 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G41" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>周邊仍有不少中小型工廠營運（需現場確認氣味/噪音影響）</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>周邊廠辦林立（土城科技園區一帶），需現場確認實際影響</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>網友指出山坡地旁有夜總會（墓地），為主要嫌惡設施疑慮
+建議現場實地確認可視範圍與距離</t>
         </is>
       </c>
       <c r="H41" s="9" t="inlineStr">
@@ -2033,7 +2156,8 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+可至新北市土壤液化/防災圖台與國土測繪圖台查詢基地座標</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -2043,7 +2167,8 @@
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+三重屬淡水河系低地，務必查詢基地淹水潛勢圖與確認社區防水閘門配置</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
@@ -2053,12 +2178,14 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢（汐止歷史上為淹水熱區，務必查詢國土測繪圖台淹水潛勢圖並向代銷確認基地墊高）</t>
+          <t>未知待查詢
+汐止為歷史淹水熱區，務必查詢基地淹水潛勢圖、確認基地墊高與地下室防水閘門</t>
         </is>
       </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+內湖部分區域屬基隆河沿岸，建議查詢台北市防災資訊網淹水潛勢圖</t>
         </is>
       </c>
     </row>
@@ -2071,32 +2198,38 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+板橋屬新北第1期已公布中級潛勢圖資（見表尾說明）確切基地</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+新店屬新北第2期已公布中級潛勢圖資（見表尾說明）</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+三重屬新北第1期已公布中級潛勢圖資（見表尾說明）</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+土城屬新北第2期已公布中級潛勢圖資（見表尾說明）</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+汐止屬新北第2期已公布中級潛勢圖資（見表尾說明）</t>
         </is>
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>未知待查詢</t>
+          <t>未知待查詢
+台北市已公布土壤液化潛勢圖資（見表尾說明）</t>
         </is>
       </c>
     </row>
@@ -2107,34 +2240,34 @@
           <t>是否位於斷層帶</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E44" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G44" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H44" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>板橋位於盆地內、不在山腳斷層線上，但距盆地西緣較近</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>新店位於盆地東南緣，不在山腳斷層線上</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>三重位於盆地西側，斷層跡經蘆洲—關渡一帶，距三重不遠，建議逐筆確認</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>土城位於盆地西南緣，不在山腳斷層線上</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>汐止位於盆地東側外緣丘陵帶，不在山腳斷層線上；惟屬山坡地，另需注意邊坡穩定</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>內湖位於盆地東北側，不在山腳斷層線上</t>
         </is>
       </c>
     </row>
@@ -2145,9 +2278,10 @@
           <t>噪音來源（鐵路／快速道路／工廠）</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>鄰近高架橋，車流噪音為已知問題
+落地窗隔音有做但仍建議現場開窗實測</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
@@ -2155,19 +2289,20 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="E45" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G45" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢（鄰新台五路主幹道，車流噪音需現場確認）</t>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>周邊中小型工廠為主要疑慮來源</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>鄰近中央路四段主幹道與廠辦區，需現場確認</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>鄰新台五路主幹道，車流噪音需現場確認
+近中山高、北二高、北宜高、環東快速道路交會帶</t>
         </is>
       </c>
       <c r="H45" s="9" t="inlineStr">
@@ -2193,9 +2328,9 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="E46" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>純住家無店面規劃，住戶出入相對單純</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
@@ -2208,9 +2343,9 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="H46" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>管理公司提供24小時飯店式管理</t>
         </is>
       </c>
     </row>
@@ -2223,39 +2358,51 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>591實價登錄：170筆成交，均價約76萬/坪</t>
+          <t>591：170筆成交，均價約76萬/坪
+5168：326筆實登，成交總價575~5,730萬，單價75~88萬/坪
+樂屋網：170筆，均價約73.7萬/坪</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>尚未開賣／預售初期，5168查詢暫無成交紀錄，未知待查詢</t>
+          <t>591：163筆實登，最新成交年月為2026年5月（民國115年）
+樂居：近一年均價約66.97萬/坪
+（本案仍在預售階段，實登筆數持續累積中）</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>591實價登錄：554筆成交，均價約67萬/坪</t>
+          <t>591：554筆成交，均價約67萬/坪
+樂居：近一年均價65.69萬/坪（301筆）
+樂屋網：596筆，均價約66萬/坪
+5168：均價約67.9萬/坪
+成交總價區間544~3,000萬；最新約66.3萬/坪</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>591實價登錄：329筆成交，均價約75萬/坪</t>
+          <t>591：329筆成交，均價約75萬/坪
+樂屋網：335筆均價79.7萬／246筆均價76.5萬
+樂居：近一年均價76.6萬/坪
+實例：2房20.7坪 單價73.9萬 總價1,526萬（無車位）；2房20.5坪 單價74.5萬 總價1,529萬（無車位）</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>各分區均價（591/5168/樂居）：
-A區約41~44萬/坪（51筆，總價600~2,390萬）
-B區約44~47萬/坪（362筆）
-C區約42~43萬/坪（173筆，總價1,060~2,270萬）
-D區約44.8~45萬/坪（628筆）
-G區約40~45萬/坪（171筆，開價45~48萬/坪）</t>
+          <t>A區：51筆，均價約41萬/坪（單價約44萬，總價600~2,390萬）
+B區：362筆，均價約46萬/坪；樂居近一年46.89萬（195筆）
+C區：173筆，近兩年均價約42.3萬/坪，實登總價1,060~2,270萬
+D區：628筆，均價約45萬/坪；樂居近一年44.72萬（318筆）
+G區：171筆，均價約40~45萬/坪（開價45~48萬/坪）</t>
         </is>
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>社區整體實登203~227筆成交
-近一年均價約83.5~92萬/坪，近6個月約91.5萬/坪
-最新成交約92.2萬/坪（部分來源顯示區間79.9~110.7萬/坪）</t>
+          <t>樂屋網：227筆成交均價約95.8萬/坪（另載224筆92萬/坪）
+5168：均價約83.5萬／88.4萬/坪
+近一年10筆成交均價約83.5萬/坪，總價區間1,165~2,990萬
+近6個月約91.5萬/坪；最新成交約92.2萬/坪
+（另有來源顯示近一年73.78萬/坪，區間差異大，議價前務必逐筆比對）</t>
         </is>
       </c>
     </row>
@@ -2271,29 +2418,32 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>十四張聯開案未來將釋出大量住宅供給，需留意中長期競爭</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>同代銷系列尚有新濠漾II(紐約公園)、新濠漾III(巴黎公園)在銷售</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+          <t>同建商系列案密集推出（II紐約公園約73~78萬/坪、III巴黎公園約82萬/坪）
+新案價高於本案，對本案二手轉售有價格支撐但也形成競爭</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>運校重劃區持續推案，短期供給量偏多</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>本案自身分期供給量大（A~G共約1,000戶以上），二手釋出量多，議價空間與轉手競爭需留意</t>
+          <t>本案自身A~G分期供給量極大（合計逾千戶）
+二手釋出量多，轉手時同社區同質競爭最為激烈</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>社區內約6戶同時銷售中（同社區競品多，可作為議價籌碼）</t>
+          <t>社區內約6戶同時銷售中，可作為議價籌碼
+周邊新建案數未知待查詢</t>
         </is>
       </c>
     </row>
@@ -2313,35 +2463,40 @@
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>約988萬元起，戶價988~2800萬元</t>
+          <t>開價總價1,088~2,800萬
+實登成交總價575~5,730萬（含車位與大坪數戶）</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>約999~2379萬元</t>
-        </is>
-      </c>
-      <c r="E50" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+          <t>開價總價999~2,379萬
+1房（16~18坪）約落在999~1,260萬區間</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>實登成交總價544~3,000萬
+以最小戶21.79坪×66萬計約1,438萬</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>開價約1,200~2,264萬/戶</t>
+          <t>開價總價896~2,535萬（另載1,200~2,264萬/戶）
+1房12~15坪推估約896~1,150萬</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>【看屋範圍推估】以1房20坪、2房23~25坪 × 均價42~46萬/坪計
-1房約840~920萬、2房約970~1,150萬
-（實際開價需向代銷確認，A區實登總價下緣約600萬）</t>
+          <t>廣告訴求總價880萬起
+【看屋範圍推估】1房20坪×約45萬≈900萬；2房23~25坪×約45萬≈1,035~1,125萬
+A區實登總價下緣約600萬</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
           <t>【看屋範圍】1房（1房0廳1衛）最低總價約1,165萬元起
-（早期首購開價約950萬起，現行行情已高於此）</t>
+社區整體成交總價1,165~2,990萬
+（早期首購開價約950萬起，現行行情已明顯高於此）</t>
         </is>
       </c>
     </row>
@@ -2354,33 +2509,38 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>開價75~88萬/坪（近期實登均價約76萬/坪）</t>
+          <t>開價75~88萬/坪
+實際成交約73.7~76萬/坪</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>開價約59~70萬/坪</t>
+          <t>開價59~70萬/坪
+實際成交近一年約66.97萬/坪</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>開價約51~65萬/坪（不同時期資料略有差異）</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+          <t>成交約65.7~67.9萬/坪
+開價曾為51~65萬/坪（早期）</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>開價68~85萬/坪
+實際成交約73.9~79.7萬/坪</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>成交約40~47萬/坪（依分區與屋齡不同）
-G區開價45~48萬/坪</t>
+          <t>各分區成交約40~47萬/坪
+G區開價45~48萬/坪為全案最高</t>
         </is>
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>約83.5~92萬/坪（近期成交），早期開價約70~85萬/坪</t>
+          <t>近期成交約83.5~92萬/坪（部分來源區間79.9~110.7萬/坪）
+早期開價約70~85萬/坪</t>
         </is>
       </c>
     </row>
@@ -2391,35 +2551,35 @@
           <t>貸款成數與利率試算</t>
         </is>
       </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H52" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢
-（小坪數套房型銀行貸款成數常低於一般住宅，務必先行詢價）</t>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>以總價1,088萬（最小戶）計：貸8成870萬，月付約3.4萬（2.5%）／約3.1萬（新青安1.775%）</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>以總價999萬（1房最小戶）計：貸8成799萬，月付約3.16萬（2.5%）／約2.86萬（新青安1.775%）</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>以總價1,438萬（最小戶21.79坪）計：貸8成1,150萬，月付約4.54萬（2.5%）／新青安僅1,000萬額度內適用</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>以總價896萬（1房最小戶）計：貸8成717萬，月付約2.83萬（2.5%）／約2.57萬（新青安1.775%）</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>以總價900萬（1房20坪）計：貸8成720萬，月付約2.84萬（2.5%）／約2.58萬（新青安1.775%）</t>
+        </is>
+      </c>
+      <c r="H52" s="8" t="inlineStr">
+        <is>
+          <t>以總價1,165萬計：貸8成932萬，月付約3.68萬（2.5%）／約3.34萬（新青安1.775%）
+⚠️小坪數套房型銀行貸款成數常低於8成（可能僅6~7成），務必先行詢價</t>
         </is>
       </c>
     </row>
@@ -2430,34 +2590,40 @@
           <t>頭期款與付款方式（工程期款）</t>
         </is>
       </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E53" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>新成屋：頭期約2成約218萬（以1,088萬計）+ 稅費
+實際付款方式需向代銷確認</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>預售屋：訂簽開約10~15%、工程期款分期、交屋款
+以999萬計頭期約2成200萬，實際成數需向代銷確認</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>已完工社區為一次性買賣
+以1,438萬計頭期約2成288萬 + 稅費</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>預售屋：訂簽開＋工程期款分期＋交屋款
+以896萬計頭期約2成179萬，實際成數需向代銷確認</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>建商宣傳「首付58萬起」（需向代銷確認適用房型與付款條件）</t>
+          <t>建商宣傳「首付58萬起」（需向代銷確認適用房型與付款條件）
+以900萬計一般頭期約2成180萬</t>
         </is>
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>已完工新古屋，為一次性買賣非工程期款；頭期款依貸款成數而定，未知待查詢</t>
+          <t>已完工成屋，為一次性買賣非工程期款
+以1,165萬、貸8成計頭期約233萬；若僅核貸7成則需350萬</t>
         </is>
       </c>
     </row>
@@ -2468,34 +2634,34 @@
           <t>稅費估算（契稅／印花稅／代書費）</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G54" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H54" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>以1,088萬計約11~16萬</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>以999萬計約10~15萬</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>以1,438萬計約14~22萬</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>以896萬計約9~13萬</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>以900萬計約9~14萬</t>
+        </is>
+      </c>
+      <c r="H54" s="8" t="inlineStr">
+        <is>
+          <t>以1,165萬計約12~17萬（中古屋另有仲介服務費，買方約成交價1~2%約12~23萬）</t>
         </is>
       </c>
     </row>
@@ -2526,14 +2692,17 @@
           <t>未知待查詢</t>
         </is>
       </c>
-      <c r="G55" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="H55" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>B區、D區均為80元/坪/月
+以1房20坪計約1,600元/月；2房25坪約2,000元/月
+A/C/G區未知待查詢</t>
+        </is>
+      </c>
+      <c r="H55" s="8" t="inlineStr">
+        <is>
+          <t>約140元/坪/月（24小時飯店式管理）
+以12坪計約1,680元/月；18坪約2,520元/月</t>
         </is>
       </c>
     </row>
@@ -2544,35 +2713,41 @@
           <t>增值潛力／轉手性評估</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="D56" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢</t>
-        </is>
-      </c>
-      <c r="G56" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢（本案量體大、同社區釋出戶數多，轉手時同質競爭激烈，須實地評估）</t>
-        </is>
-      </c>
-      <c r="H56" s="9" t="inlineStr">
-        <is>
-          <t>未知待查詢
-注意：完工年份資料分歧（一說2019年7月、一說2022年），屋齡影響貸款與轉手，請向房仲索取謄本確認</t>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>雙捷交匯與新埔成熟商圈為支撐
+但公設比近40%、高架橋噪音為轉手時的議價點</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>利多：三捷交會、十四張聯開案題材
+風險：預售價已達66~70萬/坪，短期補漲空間需觀察</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>同系列新案價位已達73~82萬/坪，對本案（約66萬）具比價支撐
+但最小戶21.79坪、總價已破1,400萬，非低總價產品</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>利多：頂埔站步行可及、三鶯線通車、土城科技園區就業支撐、四大標章
+風險：661戶大量體＋重劃區供給多，轉手同質競爭激烈</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>利多：基隆捷運保長坑2號站距基地約350公尺（環評中）
+風險：無現有捷運、量體逾千戶、汐止淹水與濕氣印象、鄰近墓地，轉手議價空間需預留</t>
+        </is>
+      </c>
+      <c r="H56" s="8" t="inlineStr">
+        <is>
+          <t>利多：北市門牌、內科就業支撐、捷運與機能成熟、租賃需求強
+風險：公設比39%、機械車位、小坪數貸款成數受限
+⚠️完工年份資料分歧（2019年7月／2022年／屋齡約2年三種說法），屋齡直接影響貸款與轉手，務必向房仲索取謄本確認</t>
         </is>
       </c>
     </row>

</xml_diff>